<commit_message>
Remove project authorship dates (data as-of dates unchanged)
</commit_message>
<xml_diff>
--- a/ADBE_3statement_model.xlsx
+++ b/ADBE_3statement_model.xlsx
@@ -22,9 +22,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="5">
-    <numFmt numFmtId="164" formatCode="#,##0.0"/>
-    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="#,##0.0"/>
     <numFmt numFmtId="167" formatCode="0.0&quot;x&quot;"/>
     <numFmt numFmtId="168" formatCode="0.000"/>
   </numFmts>
@@ -106,33 +106,42 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -522,7 +531,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Archit Chawla · October 20, 2026 · All figures from SEC EDGAR filings unless noted; $ in millions except per-share</t>
+          <t>Archit Chawla · All figures from SEC EDGAR filings unless noted; $ in millions except per-share</t>
         </is>
       </c>
     </row>
@@ -546,7 +555,7 @@
           <t>Target price</t>
         </is>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="26">
         <f>Valuation!$B$37</f>
         <v/>
       </c>
@@ -557,7 +566,7 @@
           <t>Price (close, Oct 19, 2026)</t>
         </is>
       </c>
-      <c r="B8" s="6">
+      <c r="B8" s="27">
         <f>Assumptions!$B$5</f>
         <v/>
       </c>
@@ -568,7 +577,7 @@
           <t>Implied upside</t>
         </is>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="28">
         <f>Valuation!$B$39</f>
         <v/>
       </c>
@@ -631,7 +640,7 @@
           <t>Shares outstanding (Sep 18, 2026)</t>
         </is>
       </c>
-      <c r="B16" s="9">
+      <c r="B16" s="29">
         <f>Assumptions!$B$6</f>
         <v/>
       </c>
@@ -1228,28 +1237,28 @@
           <t>WeightedAverageNumberOfDilutedSharesOutstanding (9M = mean of quarters)</t>
         </is>
       </c>
-      <c r="C17" s="9" t="n">
+      <c r="C17" s="29" t="n">
         <v>481</v>
       </c>
-      <c r="D17" s="9" t="n">
+      <c r="D17" s="29" t="n">
         <v>470.9</v>
       </c>
-      <c r="E17" s="9" t="n">
+      <c r="E17" s="29" t="n">
         <v>459.1</v>
       </c>
-      <c r="F17" s="9" t="n">
+      <c r="F17" s="29" t="n">
         <v>449.7</v>
       </c>
-      <c r="G17" s="9" t="n">
+      <c r="G17" s="29" t="n">
         <v>427</v>
       </c>
-      <c r="H17" s="9" t="n">
+      <c r="H17" s="29" t="n">
         <v>430.2</v>
       </c>
-      <c r="I17" s="9" t="n">
+      <c r="I17" s="29" t="n">
         <v>402.9</v>
       </c>
-      <c r="J17" s="9">
+      <c r="J17" s="29">
         <f>G17</f>
         <v/>
       </c>
@@ -1260,35 +1269,35 @@
           <t>Diluted EPS (GAAP)</t>
         </is>
       </c>
-      <c r="C18" s="6">
+      <c r="C18" s="27">
         <f>C16/C17</f>
         <v/>
       </c>
-      <c r="D18" s="6">
+      <c r="D18" s="27">
         <f>D16/D17</f>
         <v/>
       </c>
-      <c r="E18" s="6">
+      <c r="E18" s="27">
         <f>E16/E17</f>
         <v/>
       </c>
-      <c r="F18" s="6">
+      <c r="F18" s="27">
         <f>F16/F17</f>
         <v/>
       </c>
-      <c r="G18" s="6">
+      <c r="G18" s="27">
         <f>G16/G17</f>
         <v/>
       </c>
-      <c r="H18" s="6">
+      <c r="H18" s="27">
         <f>H16/H17</f>
         <v/>
       </c>
-      <c r="I18" s="6">
+      <c r="I18" s="27">
         <f>I16/I17</f>
         <v/>
       </c>
-      <c r="J18" s="6">
+      <c r="J18" s="27">
         <f>J16/J17</f>
         <v/>
       </c>
@@ -1868,16 +1877,16 @@
           <t>dei EntityCommonStockSharesOutstanding — 10-K cover dates for FY23–FY25; Q3 FY26 10-Q cover (Sep 18, 2026) in Latest column</t>
         </is>
       </c>
-      <c r="E38" s="9" t="n">
+      <c r="E38" s="29" t="n">
         <v>452</v>
       </c>
-      <c r="F38" s="9" t="n">
+      <c r="F38" s="29" t="n">
         <v>435.3</v>
       </c>
-      <c r="G38" s="9" t="n">
+      <c r="G38" s="29" t="n">
         <v>410.5</v>
       </c>
-      <c r="K38" s="9" t="n">
+      <c r="K38" s="29" t="n">
         <v>389.2</v>
       </c>
     </row>
@@ -1939,7 +1948,7 @@
           <t>Share price — close, Mon Oct 19, 2026 ($)</t>
         </is>
       </c>
-      <c r="B5" s="15" t="n">
+      <c r="B5" s="30" t="n">
         <v>247.09</v>
       </c>
       <c r="C5" t="inlineStr">
@@ -1954,7 +1963,7 @@
           <t>Shares outstanding (M) — Sep 18, 2026</t>
         </is>
       </c>
-      <c r="B6" s="16" t="n">
+      <c r="B6" s="31" t="n">
         <v>389.2</v>
       </c>
       <c r="C6" t="inlineStr">
@@ -2019,7 +2028,7 @@
         <f>Historicals!G5-Historicals!H5</f>
         <v/>
       </c>
-      <c r="C11" s="18" t="n">
+      <c r="C11" s="32" t="n">
         <v>0.12</v>
       </c>
       <c r="D11" s="8">
@@ -2042,7 +2051,7 @@
         <f>Historicals!G6-Historicals!H6</f>
         <v/>
       </c>
-      <c r="C12" s="18" t="n">
+      <c r="C12" s="32" t="n">
         <v>0.13</v>
       </c>
       <c r="D12" s="8">
@@ -2065,7 +2074,7 @@
         <f>Historicals!G8-Historicals!H8</f>
         <v/>
       </c>
-      <c r="C13" s="18" t="n">
+      <c r="C13" s="32" t="n">
         <v>0.12</v>
       </c>
       <c r="D13" s="8">
@@ -2088,7 +2097,7 @@
         <f>Historicals!G9-Historicals!H9</f>
         <v/>
       </c>
-      <c r="C14" s="18" t="n">
+      <c r="C14" s="32" t="n">
         <v>0.11</v>
       </c>
       <c r="D14" s="8">
@@ -2111,7 +2120,7 @@
         <f>Historicals!G10-Historicals!H10</f>
         <v/>
       </c>
-      <c r="C15" s="18" t="n">
+      <c r="C15" s="32" t="n">
         <v>0.05</v>
       </c>
       <c r="D15" s="8">
@@ -2244,7 +2253,7 @@
           <t>Q4 FY26E effective tax rate</t>
         </is>
       </c>
-      <c r="B22" s="18" t="n">
+      <c r="B22" s="32" t="n">
         <v>0.19</v>
       </c>
       <c r="C22" t="inlineStr">
@@ -2259,7 +2268,7 @@
           <t>Q4 FY26E diluted shares (M)</t>
         </is>
       </c>
-      <c r="B23" s="16" t="n">
+      <c r="B23" s="31" t="n">
         <v>383</v>
       </c>
       <c r="C23" t="inlineStr">
@@ -2303,13 +2312,13 @@
           <t>Trade receivables, % of revenue</t>
         </is>
       </c>
-      <c r="B27" s="18" t="n">
+      <c r="B27" s="32" t="n">
         <v>0.097</v>
       </c>
-      <c r="C27" s="18" t="n">
+      <c r="C27" s="32" t="n">
         <v>0.097</v>
       </c>
-      <c r="D27" s="18" t="n">
+      <c r="D27" s="32" t="n">
         <v>0.097</v>
       </c>
       <c r="E27" t="inlineStr">
@@ -2324,13 +2333,13 @@
           <t>Deferred revenue (current) growth</t>
         </is>
       </c>
-      <c r="B28" s="18" t="n">
+      <c r="B28" s="32" t="n">
         <v>0.1</v>
       </c>
-      <c r="C28" s="18" t="n">
+      <c r="C28" s="32" t="n">
         <v>0.1</v>
       </c>
-      <c r="D28" s="18" t="n">
+      <c r="D28" s="32" t="n">
         <v>0.1</v>
       </c>
       <c r="E28" t="inlineStr">
@@ -2378,13 +2387,13 @@
           <t>Average repurchase price ($)</t>
         </is>
       </c>
-      <c r="B31" s="15" t="n">
+      <c r="B31" s="30" t="n">
         <v>265</v>
       </c>
-      <c r="C31" s="15" t="n">
+      <c r="C31" s="30" t="n">
         <v>300</v>
       </c>
-      <c r="D31" s="15" t="n">
+      <c r="D31" s="30" t="n">
         <v>340</v>
       </c>
       <c r="E31" t="inlineStr">
@@ -2399,13 +2408,13 @@
           <t>Shares issued for equity comp (M)</t>
         </is>
       </c>
-      <c r="B32" s="16" t="n">
+      <c r="B32" s="31" t="n">
         <v>6</v>
       </c>
-      <c r="C32" s="16" t="n">
+      <c r="C32" s="31" t="n">
         <v>6</v>
       </c>
-      <c r="D32" s="16" t="n">
+      <c r="D32" s="31" t="n">
         <v>6</v>
       </c>
       <c r="E32" t="inlineStr">
@@ -2420,10 +2429,10 @@
           <t>Revenue growth</t>
         </is>
       </c>
-      <c r="C33" s="18" t="n">
+      <c r="C33" s="32" t="n">
         <v>0.11</v>
       </c>
-      <c r="D33" s="18" t="n">
+      <c r="D33" s="32" t="n">
         <v>0.105</v>
       </c>
       <c r="E33" t="inlineStr">
@@ -2438,10 +2447,10 @@
           <t>Gross margin</t>
         </is>
       </c>
-      <c r="C34" s="18" t="n">
+      <c r="C34" s="32" t="n">
         <v>0.892</v>
       </c>
-      <c r="D34" s="18" t="n">
+      <c r="D34" s="32" t="n">
         <v>0.893</v>
       </c>
       <c r="E34" t="inlineStr">
@@ -2456,10 +2465,10 @@
           <t>R&amp;D, % of revenue</t>
         </is>
       </c>
-      <c r="C35" s="18" t="n">
+      <c r="C35" s="32" t="n">
         <v>0.18</v>
       </c>
-      <c r="D35" s="18" t="n">
+      <c r="D35" s="32" t="n">
         <v>0.179</v>
       </c>
       <c r="E35" t="inlineStr">
@@ -2474,10 +2483,10 @@
           <t>Sales &amp; marketing, % of revenue</t>
         </is>
       </c>
-      <c r="C36" s="18" t="n">
+      <c r="C36" s="32" t="n">
         <v>0.27</v>
       </c>
-      <c r="D36" s="18" t="n">
+      <c r="D36" s="32" t="n">
         <v>0.267</v>
       </c>
       <c r="E36" t="inlineStr">
@@ -2492,10 +2501,10 @@
           <t>General &amp; administrative, % of revenue</t>
         </is>
       </c>
-      <c r="C37" s="18" t="n">
+      <c r="C37" s="32" t="n">
         <v>0.068</v>
       </c>
-      <c r="D37" s="18" t="n">
+      <c r="D37" s="32" t="n">
         <v>0.067</v>
       </c>
       <c r="E37" t="inlineStr">
@@ -2528,10 +2537,10 @@
           <t>Interest rate on beginning debt</t>
         </is>
       </c>
-      <c r="C39" s="18" t="n">
+      <c r="C39" s="32" t="n">
         <v>0.041</v>
       </c>
-      <c r="D39" s="18" t="n">
+      <c r="D39" s="32" t="n">
         <v>0.041</v>
       </c>
       <c r="E39" t="inlineStr">
@@ -2546,10 +2555,10 @@
           <t>Interest yield on beginning cash &amp; STI</t>
         </is>
       </c>
-      <c r="C40" s="18" t="n">
+      <c r="C40" s="32" t="n">
         <v>0.038</v>
       </c>
-      <c r="D40" s="18" t="n">
+      <c r="D40" s="32" t="n">
         <v>0.038</v>
       </c>
       <c r="E40" t="inlineStr">
@@ -2564,10 +2573,10 @@
           <t>Effective tax rate</t>
         </is>
       </c>
-      <c r="C41" s="18" t="n">
+      <c r="C41" s="32" t="n">
         <v>0.185</v>
       </c>
-      <c r="D41" s="18" t="n">
+      <c r="D41" s="32" t="n">
         <v>0.185</v>
       </c>
       <c r="E41" t="inlineStr">
@@ -2582,10 +2591,10 @@
           <t>Stock-based compensation, % of revenue</t>
         </is>
       </c>
-      <c r="C42" s="18" t="n">
+      <c r="C42" s="32" t="n">
         <v>0.078</v>
       </c>
-      <c r="D42" s="18" t="n">
+      <c r="D42" s="32" t="n">
         <v>0.076</v>
       </c>
       <c r="E42" t="inlineStr">
@@ -2618,10 +2627,10 @@
           <t>Capital expenditures, % of revenue</t>
         </is>
       </c>
-      <c r="C44" s="18" t="n">
+      <c r="C44" s="32" t="n">
         <v>0.008</v>
       </c>
-      <c r="D44" s="18" t="n">
+      <c r="D44" s="32" t="n">
         <v>0.008</v>
       </c>
       <c r="E44" t="inlineStr">
@@ -2661,7 +2670,7 @@
           <t>Risk-free rate (10Y UST)</t>
         </is>
       </c>
-      <c r="B48" s="18" t="n">
+      <c r="B48" s="32" t="n">
         <v>0.051</v>
       </c>
       <c r="C48" t="inlineStr">
@@ -2691,7 +2700,7 @@
           <t>Equity risk premium</t>
         </is>
       </c>
-      <c r="B50" s="18" t="n">
+      <c r="B50" s="32" t="n">
         <v>0.045</v>
       </c>
       <c r="C50" t="inlineStr">
@@ -2706,7 +2715,7 @@
           <t>Cost of equity (CAPM)</t>
         </is>
       </c>
-      <c r="B51" s="20">
+      <c r="B51" s="33">
         <f>Assumptions!$B$48+Assumptions!$B$49*Assumptions!$B$50</f>
         <v/>
       </c>
@@ -2722,7 +2731,7 @@
           <t>Pre-tax cost of debt</t>
         </is>
       </c>
-      <c r="B52" s="20">
+      <c r="B52" s="33">
         <f>Assumptions!$C$39</f>
         <v/>
       </c>
@@ -2738,7 +2747,7 @@
           <t>After-tax cost of debt</t>
         </is>
       </c>
-      <c r="B53" s="20">
+      <c r="B53" s="33">
         <f>Assumptions!$B$52*(1-Assumptions!$C$41)</f>
         <v/>
       </c>
@@ -2770,7 +2779,7 @@
           <t>Weight of equity</t>
         </is>
       </c>
-      <c r="B55" s="20">
+      <c r="B55" s="33">
         <f>Assumptions!$B$54/(Assumptions!$B$54+Historicals!K37)</f>
         <v/>
       </c>
@@ -2786,7 +2795,7 @@
           <t>WACC</t>
         </is>
       </c>
-      <c r="B56" s="7">
+      <c r="B56" s="28">
         <f>Assumptions!$B$55*Assumptions!$B$51+(1-Assumptions!$B$55)*Assumptions!$B$53</f>
         <v/>
       </c>
@@ -2802,7 +2811,7 @@
           <t>Terminal growth rate</t>
         </is>
       </c>
-      <c r="B57" s="18" t="n">
+      <c r="B57" s="32" t="n">
         <v>0.03</v>
       </c>
       <c r="C57" t="inlineStr">
@@ -2824,7 +2833,7 @@
           <t>FCF growth FY2029E</t>
         </is>
       </c>
-      <c r="B60" s="18" t="n">
+      <c r="B60" s="32" t="n">
         <v>0.09</v>
       </c>
       <c r="C60" t="inlineStr">
@@ -2839,7 +2848,7 @@
           <t>FCF growth FY2030E</t>
         </is>
       </c>
-      <c r="B61" s="18" t="n">
+      <c r="B61" s="32" t="n">
         <v>0.08</v>
       </c>
       <c r="C61" t="inlineStr">
@@ -2854,7 +2863,7 @@
           <t>FCF growth FY2031E</t>
         </is>
       </c>
-      <c r="B62" s="18" t="n">
+      <c r="B62" s="32" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="C62" t="inlineStr">
@@ -2869,7 +2878,7 @@
           <t>Bear case: FCF level shock</t>
         </is>
       </c>
-      <c r="B63" s="18" t="n">
+      <c r="B63" s="32" t="n">
         <v>-0.18</v>
       </c>
       <c r="C63" t="inlineStr">
@@ -2884,10 +2893,9 @@
           <t>Bear case: WACC add-on</t>
         </is>
       </c>
-      <c r="B64" s="18" t="n">
+      <c r="B64" s="32" t="n">
         <v>0.005</v>
       </c>
-      <c r="C64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2895,10 +2903,9 @@
           <t>Bear case: terminal growth</t>
         </is>
       </c>
-      <c r="B65" s="18" t="n">
+      <c r="B65" s="32" t="n">
         <v>0.025</v>
       </c>
-      <c r="C65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2906,7 +2913,7 @@
           <t>Bull case: FCF level shock</t>
         </is>
       </c>
-      <c r="B66" s="18" t="n">
+      <c r="B66" s="32" t="n">
         <v>0.08</v>
       </c>
       <c r="C66" t="inlineStr">
@@ -2921,10 +2928,9 @@
           <t>Bull case: WACC add-on</t>
         </is>
       </c>
-      <c r="B67" s="18" t="n">
+      <c r="B67" s="32" t="n">
         <v>-0.005</v>
       </c>
-      <c r="C67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2932,10 +2938,9 @@
           <t>Bull case: terminal growth</t>
         </is>
       </c>
-      <c r="B68" s="18" t="n">
+      <c r="B68" s="32" t="n">
         <v>0.035</v>
       </c>
-      <c r="C68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2943,7 +2948,7 @@
           <t>Disruption case: WACC</t>
         </is>
       </c>
-      <c r="B69" s="18" t="n">
+      <c r="B69" s="32" t="n">
         <v>0.115</v>
       </c>
       <c r="C69" t="inlineStr">
@@ -2958,7 +2963,7 @@
           <t>Disruption case: terminal growth</t>
         </is>
       </c>
-      <c r="B70" s="18" t="n">
+      <c r="B70" s="32" t="n">
         <v>0.015</v>
       </c>
       <c r="C70" t="inlineStr">
@@ -3318,19 +3323,19 @@
           <t>Diluted weighted-average shares</t>
         </is>
       </c>
-      <c r="C17" s="9">
+      <c r="C17" s="29">
         <f>Historicals!G17</f>
         <v/>
       </c>
-      <c r="D17" s="9">
+      <c r="D17" s="29">
         <f>(Historicals!I17*9+Assumptions!$B$23*3)/12</f>
         <v/>
       </c>
-      <c r="E17" s="9">
+      <c r="E17" s="29">
         <f>'CF_BS'!E41</f>
         <v/>
       </c>
-      <c r="F17" s="9">
+      <c r="F17" s="29">
         <f>'CF_BS'!F41</f>
         <v/>
       </c>
@@ -3341,19 +3346,19 @@
           <t>Diluted EPS (GAAP)</t>
         </is>
       </c>
-      <c r="C18" s="6">
+      <c r="C18" s="27">
         <f>C16/C17</f>
         <v/>
       </c>
-      <c r="D18" s="6">
+      <c r="D18" s="27">
         <f>D16/D17</f>
         <v/>
       </c>
-      <c r="E18" s="6">
+      <c r="E18" s="27">
         <f>E16/E17</f>
         <v/>
       </c>
-      <c r="F18" s="6">
+      <c r="F18" s="27">
         <f>F16/F17</f>
         <v/>
       </c>
@@ -3364,19 +3369,19 @@
           <t>Memo: non-GAAP EPS proxy (NI + SBC + amort. of acquired intangibles, pre-tax)</t>
         </is>
       </c>
-      <c r="C19" s="6">
+      <c r="C19" s="27">
         <f>(C16+Historicals!G21+C10)/C17</f>
         <v/>
       </c>
-      <c r="D19" s="6">
+      <c r="D19" s="27">
         <f>(D16+'CF_BS'!D7+D10)/D17</f>
         <v/>
       </c>
-      <c r="E19" s="6">
+      <c r="E19" s="27">
         <f>(E16+'CF_BS'!E7+E10)/E17</f>
         <v/>
       </c>
-      <c r="F19" s="6">
+      <c r="F19" s="27">
         <f>(F16+'CF_BS'!F7+F10)/F17</f>
         <v/>
       </c>
@@ -4049,15 +4054,15 @@
           <t>Shares outstanding, beginning</t>
         </is>
       </c>
-      <c r="D37" s="9">
+      <c r="D37" s="29">
         <f>Historicals!G38</f>
         <v/>
       </c>
-      <c r="E37" s="9">
+      <c r="E37" s="29">
         <f>D40</f>
         <v/>
       </c>
-      <c r="F37" s="9">
+      <c r="F37" s="29">
         <f>E40</f>
         <v/>
       </c>
@@ -4068,15 +4073,15 @@
           <t>Less: shares repurchased</t>
         </is>
       </c>
-      <c r="D38" s="9">
+      <c r="D38" s="29">
         <f>D15/Assumptions!$B$31</f>
         <v/>
       </c>
-      <c r="E38" s="9">
+      <c r="E38" s="29">
         <f>E15/Assumptions!$C$31</f>
         <v/>
       </c>
-      <c r="F38" s="9">
+      <c r="F38" s="29">
         <f>F15/Assumptions!$D$31</f>
         <v/>
       </c>
@@ -4087,15 +4092,15 @@
           <t>Plus: shares issued for equity comp</t>
         </is>
       </c>
-      <c r="D39" s="9">
+      <c r="D39" s="29">
         <f>Assumptions!$B$32</f>
         <v/>
       </c>
-      <c r="E39" s="9">
+      <c r="E39" s="29">
         <f>Assumptions!$C$32</f>
         <v/>
       </c>
-      <c r="F39" s="9">
+      <c r="F39" s="29">
         <f>Assumptions!$D$32</f>
         <v/>
       </c>
@@ -4106,15 +4111,15 @@
           <t>Shares outstanding, end of year</t>
         </is>
       </c>
-      <c r="D40" s="23">
+      <c r="D40" s="34">
         <f>D37-D38+D39</f>
         <v/>
       </c>
-      <c r="E40" s="23">
+      <c r="E40" s="34">
         <f>E37-E38+E39</f>
         <v/>
       </c>
-      <c r="F40" s="23">
+      <c r="F40" s="34">
         <f>F37-F38+F39</f>
         <v/>
       </c>
@@ -4125,11 +4130,11 @@
           <t>Diluted weighted-average shares (BS roll)</t>
         </is>
       </c>
-      <c r="E41" s="9">
+      <c r="E41" s="29">
         <f>(E37+E40)/2</f>
         <v/>
       </c>
-      <c r="F41" s="9">
+      <c r="F41" s="29">
         <f>(F37+F40)/2</f>
         <v/>
       </c>
@@ -4647,7 +4652,7 @@
           <t>WACC</t>
         </is>
       </c>
-      <c r="B29" s="20">
+      <c r="B29" s="33">
         <f>Assumptions!$B$56</f>
         <v/>
       </c>
@@ -4658,7 +4663,7 @@
           <t>Terminal growth</t>
         </is>
       </c>
-      <c r="B30" s="20">
+      <c r="B30" s="33">
         <f>Assumptions!$B$57</f>
         <v/>
       </c>
@@ -4724,7 +4729,7 @@
           <t>Diluted shares out (M)</t>
         </is>
       </c>
-      <c r="B36" s="9">
+      <c r="B36" s="29">
         <f>Assumptions!$B$6</f>
         <v/>
       </c>
@@ -4735,7 +4740,7 @@
           <t>TARGET PRICE</t>
         </is>
       </c>
-      <c r="B37" s="5">
+      <c r="B37" s="26">
         <f>B35/B36</f>
         <v/>
       </c>
@@ -4746,7 +4751,7 @@
           <t>Current price</t>
         </is>
       </c>
-      <c r="B38" s="6">
+      <c r="B38" s="27">
         <f>Assumptions!$B$5</f>
         <v/>
       </c>
@@ -4757,7 +4762,7 @@
           <t>Implied upside</t>
         </is>
       </c>
-      <c r="B39" s="7">
+      <c r="B39" s="28">
         <f>B37/B38-1</f>
         <v/>
       </c>
@@ -4852,11 +4857,11 @@
         <f>F25</f>
         <v/>
       </c>
-      <c r="G43" s="20">
+      <c r="G43" s="33">
         <f>Valuation!$B$29</f>
         <v/>
       </c>
-      <c r="H43" s="20">
+      <c r="H43" s="33">
         <f>Valuation!$B$30</f>
         <v/>
       </c>
@@ -4864,11 +4869,11 @@
         <f>B43/(1+$G43)^1+C43/(1+$G43)^2+D43/(1+$G43)^3+E43/(1+$G43)^4+F43/(1+$G43)^5+F43*(1+H43)/(G43-H43)/(1+G43)^5-Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="J43" s="6">
+      <c r="J43" s="27">
         <f>I43/Assumptions!$B$6</f>
         <v/>
       </c>
-      <c r="K43" s="20">
+      <c r="K43" s="33">
         <f>J43/Assumptions!$B$5-1</f>
         <v/>
       </c>
@@ -4899,11 +4904,11 @@
         <f>F25*(1+Assumptions!$B$63)</f>
         <v/>
       </c>
-      <c r="G44" s="20">
+      <c r="G44" s="33">
         <f>Valuation!$B$29+Assumptions!$B$64</f>
         <v/>
       </c>
-      <c r="H44" s="20">
+      <c r="H44" s="33">
         <f>Assumptions!$B$65</f>
         <v/>
       </c>
@@ -4911,11 +4916,11 @@
         <f>B44/(1+$G44)^1+C44/(1+$G44)^2+D44/(1+$G44)^3+E44/(1+$G44)^4+F44/(1+$G44)^5+F44*(1+H44)/(G44-H44)/(1+G44)^5-Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="J44" s="6">
+      <c r="J44" s="27">
         <f>I44/Assumptions!$B$6</f>
         <v/>
       </c>
-      <c r="K44" s="20">
+      <c r="K44" s="33">
         <f>J44/Assumptions!$B$5-1</f>
         <v/>
       </c>
@@ -4946,11 +4951,11 @@
         <f>F25*(1+Assumptions!$B$66)</f>
         <v/>
       </c>
-      <c r="G45" s="20">
+      <c r="G45" s="33">
         <f>Valuation!$B$29+Assumptions!$B$67</f>
         <v/>
       </c>
-      <c r="H45" s="20">
+      <c r="H45" s="33">
         <f>Assumptions!$B$68</f>
         <v/>
       </c>
@@ -4958,11 +4963,11 @@
         <f>B45/(1+$G45)^1+C45/(1+$G45)^2+D45/(1+$G45)^3+E45/(1+$G45)^4+F45/(1+$G45)^5+F45*(1+H45)/(G45-H45)/(1+G45)^5-Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="J45" s="6">
+      <c r="J45" s="27">
         <f>I45/Assumptions!$B$6</f>
         <v/>
       </c>
-      <c r="K45" s="20">
+      <c r="K45" s="33">
         <f>J45/Assumptions!$B$5-1</f>
         <v/>
       </c>
@@ -4988,11 +4993,11 @@
       <c r="F46" s="8" t="n">
         <v>9700</v>
       </c>
-      <c r="G46" s="20">
+      <c r="G46" s="33">
         <f>Assumptions!$B$69</f>
         <v/>
       </c>
-      <c r="H46" s="20">
+      <c r="H46" s="33">
         <f>Assumptions!$B$70</f>
         <v/>
       </c>
@@ -5000,11 +5005,11 @@
         <f>B46/(1+$G46)^1+C46/(1+$G46)^2+D46/(1+$G46)^3+E46/(1+$G46)^4+F46/(1+$G46)^5+F46*(1+H46)/(G46-H46)/(1+G46)^5-Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="J46" s="6">
+      <c r="J46" s="27">
         <f>I46/Assumptions!$B$6</f>
         <v/>
       </c>
-      <c r="K46" s="20">
+      <c r="K46" s="33">
         <f>J46/Assumptions!$B$5-1</f>
         <v/>
       </c>
@@ -5024,102 +5029,102 @@
       </c>
     </row>
     <row r="50">
-      <c r="B50" s="7" t="n">
+      <c r="B50" s="28" t="n">
         <v>0.025</v>
       </c>
-      <c r="C50" s="7" t="n">
+      <c r="C50" s="28" t="n">
         <v>0.03</v>
       </c>
-      <c r="D50" s="7" t="n">
+      <c r="D50" s="28" t="n">
         <v>0.035</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="20">
+      <c r="A51" s="33">
         <f>Valuation!$B$29+-0.01</f>
         <v/>
       </c>
-      <c r="B51" s="6">
+      <c r="B51" s="27">
         <f>(B25/(1+$A51)^1+C25/(1+$A51)^2+D25/(1+$A51)^3+E25/(1+$A51)^4+F25/(1+$A51)^5+F$25*(1+B$50)/($A51-B$50)/(1+$A51)^5-Assumptions!$B$7)/Assumptions!$B$6</f>
         <v/>
       </c>
-      <c r="C51" s="6">
+      <c r="C51" s="27">
         <f>(B25/(1+$A51)^1+C25/(1+$A51)^2+D25/(1+$A51)^3+E25/(1+$A51)^4+F25/(1+$A51)^5+F$25*(1+C$50)/($A51-C$50)/(1+$A51)^5-Assumptions!$B$7)/Assumptions!$B$6</f>
         <v/>
       </c>
-      <c r="D51" s="6">
+      <c r="D51" s="27">
         <f>(B25/(1+$A51)^1+C25/(1+$A51)^2+D25/(1+$A51)^3+E25/(1+$A51)^4+F25/(1+$A51)^5+F$25*(1+D$50)/($A51-D$50)/(1+$A51)^5-Assumptions!$B$7)/Assumptions!$B$6</f>
         <v/>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="20">
+      <c r="A52" s="33">
         <f>Valuation!$B$29+-0.005</f>
         <v/>
       </c>
-      <c r="B52" s="6">
+      <c r="B52" s="27">
         <f>(B25/(1+$A52)^1+C25/(1+$A52)^2+D25/(1+$A52)^3+E25/(1+$A52)^4+F25/(1+$A52)^5+F$25*(1+B$50)/($A52-B$50)/(1+$A52)^5-Assumptions!$B$7)/Assumptions!$B$6</f>
         <v/>
       </c>
-      <c r="C52" s="6">
+      <c r="C52" s="27">
         <f>(B25/(1+$A52)^1+C25/(1+$A52)^2+D25/(1+$A52)^3+E25/(1+$A52)^4+F25/(1+$A52)^5+F$25*(1+C$50)/($A52-C$50)/(1+$A52)^5-Assumptions!$B$7)/Assumptions!$B$6</f>
         <v/>
       </c>
-      <c r="D52" s="6">
+      <c r="D52" s="27">
         <f>(B25/(1+$A52)^1+C25/(1+$A52)^2+D25/(1+$A52)^3+E25/(1+$A52)^4+F25/(1+$A52)^5+F$25*(1+D$50)/($A52-D$50)/(1+$A52)^5-Assumptions!$B$7)/Assumptions!$B$6</f>
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="20">
+      <c r="A53" s="33">
         <f>Valuation!$B$29+0.0</f>
         <v/>
       </c>
-      <c r="B53" s="6">
+      <c r="B53" s="27">
         <f>(B25/(1+$A53)^1+C25/(1+$A53)^2+D25/(1+$A53)^3+E25/(1+$A53)^4+F25/(1+$A53)^5+F$25*(1+B$50)/($A53-B$50)/(1+$A53)^5-Assumptions!$B$7)/Assumptions!$B$6</f>
         <v/>
       </c>
-      <c r="C53" s="6">
+      <c r="C53" s="27">
         <f>(B25/(1+$A53)^1+C25/(1+$A53)^2+D25/(1+$A53)^3+E25/(1+$A53)^4+F25/(1+$A53)^5+F$25*(1+C$50)/($A53-C$50)/(1+$A53)^5-Assumptions!$B$7)/Assumptions!$B$6</f>
         <v/>
       </c>
-      <c r="D53" s="6">
+      <c r="D53" s="27">
         <f>(B25/(1+$A53)^1+C25/(1+$A53)^2+D25/(1+$A53)^3+E25/(1+$A53)^4+F25/(1+$A53)^5+F$25*(1+D$50)/($A53-D$50)/(1+$A53)^5-Assumptions!$B$7)/Assumptions!$B$6</f>
         <v/>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="20">
+      <c r="A54" s="33">
         <f>Valuation!$B$29+0.005</f>
         <v/>
       </c>
-      <c r="B54" s="6">
+      <c r="B54" s="27">
         <f>(B25/(1+$A54)^1+C25/(1+$A54)^2+D25/(1+$A54)^3+E25/(1+$A54)^4+F25/(1+$A54)^5+F$25*(1+B$50)/($A54-B$50)/(1+$A54)^5-Assumptions!$B$7)/Assumptions!$B$6</f>
         <v/>
       </c>
-      <c r="C54" s="6">
+      <c r="C54" s="27">
         <f>(B25/(1+$A54)^1+C25/(1+$A54)^2+D25/(1+$A54)^3+E25/(1+$A54)^4+F25/(1+$A54)^5+F$25*(1+C$50)/($A54-C$50)/(1+$A54)^5-Assumptions!$B$7)/Assumptions!$B$6</f>
         <v/>
       </c>
-      <c r="D54" s="6">
+      <c r="D54" s="27">
         <f>(B25/(1+$A54)^1+C25/(1+$A54)^2+D25/(1+$A54)^3+E25/(1+$A54)^4+F25/(1+$A54)^5+F$25*(1+D$50)/($A54-D$50)/(1+$A54)^5-Assumptions!$B$7)/Assumptions!$B$6</f>
         <v/>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="20">
+      <c r="A55" s="33">
         <f>Valuation!$B$29+0.01</f>
         <v/>
       </c>
-      <c r="B55" s="6">
+      <c r="B55" s="27">
         <f>(B25/(1+$A55)^1+C25/(1+$A55)^2+D25/(1+$A55)^3+E25/(1+$A55)^4+F25/(1+$A55)^5+F$25*(1+B$50)/($A55-B$50)/(1+$A55)^5-Assumptions!$B$7)/Assumptions!$B$6</f>
         <v/>
       </c>
-      <c r="C55" s="6">
+      <c r="C55" s="27">
         <f>(B25/(1+$A55)^1+C25/(1+$A55)^2+D25/(1+$A55)^3+E25/(1+$A55)^4+F25/(1+$A55)^5+F$25*(1+C$50)/($A55-C$50)/(1+$A55)^5-Assumptions!$B$7)/Assumptions!$B$6</f>
         <v/>
       </c>
-      <c r="D55" s="6">
+      <c r="D55" s="27">
         <f>(B25/(1+$A55)^1+C25/(1+$A55)^2+D25/(1+$A55)^3+E25/(1+$A55)^4+F25/(1+$A55)^5+F$25*(1+D$50)/($A55-D$50)/(1+$A55)^5-Assumptions!$B$7)/Assumptions!$B$6</f>
         <v/>
       </c>
@@ -5137,7 +5142,7 @@
           <t>FY27E FCF per share</t>
         </is>
       </c>
-      <c r="B58" s="6">
+      <c r="B58" s="27">
         <f>'CF_BS'!E13/IS!E17</f>
         <v/>
       </c>
@@ -5148,7 +5153,7 @@
           <t>Implied price at FY25's own (already de-rated) P/FCF</t>
         </is>
       </c>
-      <c r="B59" s="6">
+      <c r="B59" s="27">
         <f>Valuation!$H$20*Valuation!$B$58</f>
         <v/>
       </c>
@@ -5159,7 +5164,7 @@
           <t>FY27E GAAP EPS</t>
         </is>
       </c>
-      <c r="B60" s="6">
+      <c r="B60" s="27">
         <f>IS!E18</f>
         <v/>
       </c>
@@ -5170,7 +5175,7 @@
           <t>Implied price at 20.0× FY27E GAAP EPS</t>
         </is>
       </c>
-      <c r="B61" s="6">
+      <c r="B61" s="27">
         <f>B60*20</f>
         <v/>
       </c>

</xml_diff>